<commit_message>
Changes the priority of the XBRL facts for the Long Term Debt metric to more reliably pull the correct non-current value across the airlines. The re-order better handles differences in reporting. Data reloaded using the corrected fact priority and DAL 2026Q3 results added.
</commit_message>
<xml_diff>
--- a/airline-dashboard/data/manual/airline_financial_data.xlsx
+++ b/airline-dashboard/data/manual/airline_financial_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/GitHub Repos/airline_financials/airline-dashboard/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5F27149-13F5-42E4-A5A1-626E2D31AE68}"/>
+  <xr:revisionPtr revIDLastSave="187" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C001F13-96BC-49F2-90EC-00B5CCF364B1}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
   <sheets>
     <sheet name="airline_financials" sheetId="2" r:id="rId1"/>
@@ -997,7 +997,7 @@
     <col min="8" max="9" width="17.140625" customWidth="1"/>
     <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -12653,9 +12653,9 @@
       <c r="J505">
         <v>27853000000</v>
       </c>
-      <c r="K505" t="e">
-        <f>ROUND($K$219*((D505-F505)/($D$219-$F$219)),0)</f>
-        <v>#DIV/0!</v>
+      <c r="K505">
+        <f>ROUND($K$547*((D505-F505)/($D$547-$F$547)),0)</f>
+        <v>610559</v>
       </c>
     </row>
     <row r="506" spans="1:11" x14ac:dyDescent="0.25">
@@ -12910,9 +12910,9 @@
       <c r="J516">
         <v>27209000000</v>
       </c>
-      <c r="K516" t="e">
-        <f>ROUND($K$219*((D516-F516)/($D$219-$F$219)),0)</f>
-        <v>#DIV/0!</v>
+      <c r="K516">
+        <f>ROUND($K$547*((D516-F516)/($D$547-$F$547)),0)</f>
+        <v>120716144</v>
       </c>
     </row>
     <row r="517" spans="1:11" x14ac:dyDescent="0.25">
@@ -13167,9 +13167,9 @@
       <c r="J527">
         <v>25848000000</v>
       </c>
-      <c r="K527" t="e">
-        <f>ROUND($K$219*((D527-F527)/($D$219-$F$219)),0)</f>
-        <v>#DIV/0!</v>
+      <c r="K527">
+        <f>ROUND($K$547*((D527-F527)/($D$547-$F$547)),0)</f>
+        <v>7762816</v>
       </c>
     </row>
     <row r="528" spans="1:11" x14ac:dyDescent="0.25">
@@ -13407,9 +13407,9 @@
       <c r="J537">
         <v>24617000000</v>
       </c>
-      <c r="K537" t="e">
-        <f>ROUND($K$219*((D537-F537)/($D$219-$F$219)),0)</f>
-        <v>#DIV/0!</v>
+      <c r="K537">
+        <f>ROUND($K$547*((D537-F537)/($D$547-$F$547)),0)</f>
+        <v>98910482</v>
       </c>
     </row>
     <row r="538" spans="1:11" x14ac:dyDescent="0.25">
@@ -13893,6 +13893,7 @@
         <v>24705000000</v>
       </c>
       <c r="K557">
+        <f>IF(D557-F557&gt;0, ROUND($K$597*((D557-F557)/(IF(($D$557-$F$557)&gt;0, ($D$557-$F$557), 0)+IF(($D$567-$F$567)&gt;0, ($D$567-$F$567), 0)+IF(($D$577-$F$577)&gt;0, ($D$577-$F$577), 0)+IF(($D$587-$F$587)&gt;0, ($D$587-$F$587), 0))),0), 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -14132,7 +14133,8 @@
         <v>24217000000</v>
       </c>
       <c r="K567">
-        <v>41000000</v>
+        <f>IF(D567-F567&gt;0, ROUND($K$597*((D567-F567)/(IF(($D$557-$F$557)&gt;0, ($D$557-$F$557), 0)+IF(($D$567-$F$567)&gt;0, ($D$567-$F$567), 0)+IF(($D$577-$F$577)&gt;0, ($D$577-$F$577), 0)+IF(($D$587-$F$587)&gt;0, ($D$587-$F$587), 0))),0), 0)</f>
+        <v>35938400</v>
       </c>
     </row>
     <row r="568" spans="1:11" x14ac:dyDescent="0.25">
@@ -14371,7 +14373,8 @@
         <v>24538000000</v>
       </c>
       <c r="K577">
-        <v>0</v>
+        <f>IF(D577-F577&gt;0, ROUND($K$597*((D577-F577)/(IF(($D$557-$F$557)&gt;0, ($D$557-$F$557), 0)+IF(($D$567-$F$567)&gt;0, ($D$567-$F$567), 0)+IF(($D$577-$F$577)&gt;0, ($D$577-$F$577), 0)+IF(($D$587-$F$587)&gt;0, ($D$587-$F$587), 0))),0), 0)</f>
+        <v>4781232</v>
       </c>
     </row>
     <row r="578" spans="1:11" x14ac:dyDescent="0.25">
@@ -14609,9 +14612,9 @@
       <c r="J587">
         <v>24639000000</v>
       </c>
-      <c r="K587" t="e">
-        <f>ROUND($K$241*(((D587-F587)/($D$241-$F$241))/(((D587-F587)/($D$241-$F$241))+((D575-F575)/($D$241-$F$241)))),0)</f>
-        <v>#DIV/0!</v>
+      <c r="K587">
+        <f>IF(D587-F587&gt;0, ROUND($K$597*((D587-F587)/(IF(($D$557-$F$557)&gt;0, ($D$557-$F$557), 0)+IF(($D$567-$F$567)&gt;0, ($D$567-$F$567), 0)+IF(($D$577-$F$577)&gt;0, ($D$577-$F$577), 0)+IF(($D$587-$F$587)&gt;0, ($D$587-$F$587), 0))),0), 0)</f>
+        <v>14280368</v>
       </c>
     </row>
     <row r="588" spans="1:11" x14ac:dyDescent="0.25">
@@ -15095,6 +15098,7 @@
         <v>22934000000</v>
       </c>
       <c r="K607">
+        <f>IF(D607-F607&gt;0, ROUND($K$597*((D607-F607)/(IF(($D$557-$F$557)&gt;0, ($D$557-$F$557), 0)+IF(($D$567-$F$567)&gt;0, ($D$567-$F$567), 0)+IF(($D$577-$F$577)&gt;0, ($D$577-$F$577), 0)+IF(($D$587-$F$587)&gt;0, ($D$587-$F$587), 0))),0), 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -15314,6 +15318,7 @@
         <v>81843000000</v>
       </c>
       <c r="K616">
+        <f>IF(D616-F616&gt;0, ROUND($K$640*((D616-F616)/(IF(($D$607-$F$607)&gt;0, ($D$607-$F$607), 0)+IF(($D$616-$F$616)&gt;0, ($D$616-$F$616), 0)+IF(($D$624-$F$624)&gt;0, ($D$624-$F$624), 0)+IF(($D$632-$F$632)&gt;0, ($D$632-$F$632), 0))),0), 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -15495,7 +15500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="625" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="625" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A625">
         <v>2026</v>
       </c>
@@ -15506,7 +15511,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="626" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="626" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A626">
         <v>2026</v>
       </c>
@@ -15517,7 +15522,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="627" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="627" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A627">
         <v>2026</v>
       </c>
@@ -15527,8 +15532,32 @@
       <c r="C627" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="628" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D627">
+        <v>20186000000</v>
+      </c>
+      <c r="E627">
+        <v>15534000000</v>
+      </c>
+      <c r="F627">
+        <v>18732000000</v>
+      </c>
+      <c r="G627">
+        <v>756000000</v>
+      </c>
+      <c r="H627">
+        <v>68133000000</v>
+      </c>
+      <c r="I627">
+        <v>79288000000</v>
+      </c>
+      <c r="J627">
+        <v>9124000000</v>
+      </c>
+      <c r="K627">
+        <v>389000000</v>
+      </c>
+    </row>
+    <row r="628" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A628">
         <v>2026</v>
       </c>
@@ -15539,7 +15568,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="629" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="629" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A629">
         <v>2026</v>
       </c>
@@ -15550,7 +15579,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="630" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="630" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A630">
         <v>2026</v>
       </c>
@@ -15561,7 +15590,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="631" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="631" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A631">
         <v>2026</v>
       </c>

</xml_diff>

<commit_message>
Adds LUV 2026Q3 results.
</commit_message>
<xml_diff>
--- a/airline-dashboard/data/manual/airline_financial_data.xlsx
+++ b/airline-dashboard/data/manual/airline_financial_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/GitHub Repos/airline_financials/airline-dashboard/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F546F10-6DEF-46EB-9646-2E6C2968824B}"/>
+  <xr:revisionPtr revIDLastSave="209" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E25FA96-0120-4D42-BD6D-72175F9D1F38}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
   <sheets>
     <sheet name="airline_financials" sheetId="2" r:id="rId1"/>
@@ -15614,6 +15614,9 @@
       <c r="I629">
         <v>45393000000</v>
       </c>
+      <c r="K629">
+        <v>62000000</v>
+      </c>
     </row>
     <row r="630" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A630">

</xml_diff>